<commit_message>
Add market share %, Fix District Mismatch button, EDNC subtitle
- filings.py: compute market_share % (share of tracked cases) per firm per district
- filings.html: add Share % column to all 3 district tables; add Clean PACER Dupes
  and Fix District Mismatch buttons; fix subtitle to include EDNC
- admin.py: POST /admin/clean-district-mismatch — deletes FilingSnapshot rows
  for firms in districts their markets don't map to (fixes Triad firms showing
  in WDNC with stale counts from earlier collection runs)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Competitor List.xlsx
+++ b/Competitor List.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/damonduncan/Claude-Playground/Competitor Analysis and Local SEO Intelligence Tool/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F23C192C-EE3A-294B-AAD0-E024EBA8B397}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C6D5080-C501-4145-AC05-2F5A23F0CE8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3260" yWindow="2160" windowWidth="28040" windowHeight="17440" xr2:uid="{39A3620F-FC9F-3744-B228-09DF34C1F8FA}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="270" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="280" uniqueCount="103">
   <si>
     <t>Google Place ID (search the firm at the Place ID Finder)</t>
   </si>
@@ -384,12 +384,21 @@
   <si>
     <t>https://www.bbb.org/us/nc/shelby/profile/lawyers/lutz-law-firm-0473-292619</t>
   </si>
+  <si>
+    <t>Rashad Blossom</t>
+  </si>
+  <si>
+    <t>Blossom Law PLLC</t>
+  </si>
+  <si>
+    <t>ChIJNTAcyHmfVogRsaApqMs_lMw</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="11">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -449,6 +458,17 @@
       <name val="Times New Roman"/>
       <family val="1"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Times"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -477,7 +497,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -485,6 +505,8 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -820,8 +842,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3C434DA6-306D-8346-8757-EBC8132196FB}">
-  <dimension ref="A1:Q191"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:Q197"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="101" customWidth="1"/>
     <col min="2" max="2" width="85.33203125" style="4" customWidth="1"/>
@@ -829,12 +851,12 @@
     <col min="4" max="17" width="10.83203125" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="18" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:5" ht="18">
       <c r="A1" s="3" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:5">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -842,7 +864,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:5">
       <c r="A3" s="2" t="s">
         <v>2</v>
       </c>
@@ -859,7 +881,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:5">
       <c r="A4" s="1" t="s">
         <v>0</v>
       </c>
@@ -867,7 +889,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:5">
       <c r="A5" s="2" t="s">
         <v>3</v>
       </c>
@@ -875,7 +897,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:5">
       <c r="A6" s="2" t="s">
         <v>4</v>
       </c>
@@ -883,7 +905,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:5">
       <c r="A8" s="2" t="s">
         <v>1</v>
       </c>
@@ -891,7 +913,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:5">
       <c r="A9" s="2" t="s">
         <v>2</v>
       </c>
@@ -899,7 +921,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:5">
       <c r="A10" s="1" t="s">
         <v>0</v>
       </c>
@@ -907,7 +929,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:5">
       <c r="A11" s="2" t="s">
         <v>3</v>
       </c>
@@ -915,7 +937,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:5">
       <c r="A12" s="2" t="s">
         <v>4</v>
       </c>
@@ -923,7 +945,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:5">
       <c r="A14" s="2" t="s">
         <v>1</v>
       </c>
@@ -931,7 +953,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:5">
       <c r="A15" s="2" t="s">
         <v>2</v>
       </c>
@@ -939,7 +961,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:5">
       <c r="A16" s="1" t="s">
         <v>0</v>
       </c>
@@ -947,7 +969,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:2">
       <c r="A17" s="2" t="s">
         <v>3</v>
       </c>
@@ -955,7 +977,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:2">
       <c r="A18" s="2" t="s">
         <v>4</v>
       </c>
@@ -963,7 +985,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:2">
       <c r="A20" s="2" t="s">
         <v>1</v>
       </c>
@@ -971,7 +993,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:2">
       <c r="A21" s="2" t="s">
         <v>2</v>
       </c>
@@ -979,7 +1001,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:2">
       <c r="A22" s="1" t="s">
         <v>0</v>
       </c>
@@ -987,7 +1009,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:2">
       <c r="A23" s="2" t="s">
         <v>3</v>
       </c>
@@ -995,7 +1017,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:2">
       <c r="A24" s="2" t="s">
         <v>4</v>
       </c>
@@ -1003,7 +1025,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:2">
       <c r="A26" s="2" t="s">
         <v>1</v>
       </c>
@@ -1011,7 +1033,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:2">
       <c r="A27" s="2" t="s">
         <v>2</v>
       </c>
@@ -1019,7 +1041,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:2">
       <c r="A28" s="1" t="s">
         <v>0</v>
       </c>
@@ -1027,12 +1049,12 @@
         <v>33</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:2">
       <c r="A29" s="2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:2">
       <c r="A30" s="2" t="s">
         <v>4</v>
       </c>
@@ -1040,12 +1062,12 @@
         <v>40</v>
       </c>
     </row>
-    <row r="32" spans="1:2" ht="18" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:2" ht="18">
       <c r="A32" s="3" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:2">
       <c r="A33" s="2" t="s">
         <v>1</v>
       </c>
@@ -1053,7 +1075,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:2">
       <c r="A34" s="2" t="s">
         <v>2</v>
       </c>
@@ -1061,7 +1083,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:2">
       <c r="A35" s="1" t="s">
         <v>0</v>
       </c>
@@ -1069,7 +1091,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:2">
       <c r="A36" s="2" t="s">
         <v>3</v>
       </c>
@@ -1077,7 +1099,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:2">
       <c r="A37" s="2" t="s">
         <v>4</v>
       </c>
@@ -1085,7 +1107,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:2">
       <c r="A39" s="2" t="s">
         <v>1</v>
       </c>
@@ -1093,7 +1115,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:2">
       <c r="A40" s="2" t="s">
         <v>2</v>
       </c>
@@ -1101,7 +1123,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:2">
       <c r="A41" s="1" t="s">
         <v>0</v>
       </c>
@@ -1109,7 +1131,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:2">
       <c r="A42" s="2" t="s">
         <v>3</v>
       </c>
@@ -1117,7 +1139,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:2">
       <c r="A43" s="2" t="s">
         <v>4</v>
       </c>
@@ -1125,7 +1147,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:2">
       <c r="A45" s="2" t="s">
         <v>1</v>
       </c>
@@ -1133,7 +1155,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:2">
       <c r="A46" s="2" t="s">
         <v>2</v>
       </c>
@@ -1141,7 +1163,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:2">
       <c r="A47" s="1" t="s">
         <v>0</v>
       </c>
@@ -1149,7 +1171,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:2">
       <c r="A48" s="2" t="s">
         <v>3</v>
       </c>
@@ -1157,7 +1179,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:2">
       <c r="A49" s="2" t="s">
         <v>4</v>
       </c>
@@ -1165,7 +1187,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:2">
       <c r="A51" s="2" t="s">
         <v>1</v>
       </c>
@@ -1173,7 +1195,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:2">
       <c r="A52" s="2" t="s">
         <v>2</v>
       </c>
@@ -1181,7 +1203,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:2">
       <c r="A53" s="1" t="s">
         <v>0</v>
       </c>
@@ -1189,7 +1211,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:2">
       <c r="A54" s="2" t="s">
         <v>3</v>
       </c>
@@ -1197,7 +1219,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:2">
       <c r="A55" s="2" t="s">
         <v>4</v>
       </c>
@@ -1205,37 +1227,37 @@
         <v>41</v>
       </c>
     </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:2">
       <c r="A57" s="2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:2">
       <c r="A58" s="2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:2">
       <c r="A59" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:2">
       <c r="A60" s="2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:2">
       <c r="A61" s="2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="63" spans="1:2" ht="18" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:2" ht="18">
       <c r="A63" s="3" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="64" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:2">
       <c r="A64" s="2" t="s">
         <v>1</v>
       </c>
@@ -1243,7 +1265,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:2">
       <c r="A65" s="2" t="s">
         <v>2</v>
       </c>
@@ -1251,7 +1273,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:2">
       <c r="A66" s="1" t="s">
         <v>0</v>
       </c>
@@ -1259,7 +1281,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:2">
       <c r="A67" s="2" t="s">
         <v>3</v>
       </c>
@@ -1267,7 +1289,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="68" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:2">
       <c r="A68" s="2" t="s">
         <v>4</v>
       </c>
@@ -1275,112 +1297,112 @@
         <v>40</v>
       </c>
     </row>
-    <row r="70" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:2">
       <c r="A70" s="2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="71" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:2">
       <c r="A71" s="2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="72" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:2">
       <c r="A72" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:2">
       <c r="A73" s="2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="74" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:2">
       <c r="A74" s="2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="76" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:2">
       <c r="A76" s="2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="77" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:2">
       <c r="A77" s="2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="78" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:2">
       <c r="A78" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:2">
       <c r="A79" s="2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="80" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:2">
       <c r="A80" s="2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="82" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:2">
       <c r="A82" s="2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="83" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:2">
       <c r="A83" s="2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="84" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:2">
       <c r="A84" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="85" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:2">
       <c r="A85" s="2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="86" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:2">
       <c r="A86" s="2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="88" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:2">
       <c r="A88" s="2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="89" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:2">
       <c r="A89" s="2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="90" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:2">
       <c r="A90" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="91" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:2">
       <c r="A91" s="2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="92" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:2">
       <c r="A92" s="2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="94" spans="1:2" ht="18" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:2" ht="18">
       <c r="A94" s="3" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="95" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:2">
       <c r="A95" s="2" t="s">
         <v>1</v>
       </c>
@@ -1388,7 +1410,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="96" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:2">
       <c r="A96" s="2" t="s">
         <v>2</v>
       </c>
@@ -1396,7 +1418,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="97" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:2">
       <c r="A97" s="1" t="s">
         <v>0</v>
       </c>
@@ -1404,7 +1426,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="98" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:2">
       <c r="A98" s="2" t="s">
         <v>3</v>
       </c>
@@ -1412,7 +1434,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="99" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:2">
       <c r="A99" s="2" t="s">
         <v>4</v>
       </c>
@@ -1420,7 +1442,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="101" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:2">
       <c r="A101" s="2" t="s">
         <v>1</v>
       </c>
@@ -1428,7 +1450,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="102" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:2">
       <c r="A102" s="2" t="s">
         <v>2</v>
       </c>
@@ -1436,7 +1458,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="103" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:2">
       <c r="A103" s="1" t="s">
         <v>0</v>
       </c>
@@ -1444,7 +1466,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="104" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:2">
       <c r="A104" s="2" t="s">
         <v>3</v>
       </c>
@@ -1452,7 +1474,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="105" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:2">
       <c r="A105" s="2" t="s">
         <v>4</v>
       </c>
@@ -1460,7 +1482,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="107" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:2">
       <c r="A107" s="2" t="s">
         <v>1</v>
       </c>
@@ -1468,7 +1490,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="108" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:2">
       <c r="A108" s="2" t="s">
         <v>2</v>
       </c>
@@ -1476,7 +1498,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="109" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:2">
       <c r="A109" s="1" t="s">
         <v>0</v>
       </c>
@@ -1484,7 +1506,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="110" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:2">
       <c r="A110" s="2" t="s">
         <v>3</v>
       </c>
@@ -1492,7 +1514,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="111" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:2">
       <c r="A111" s="2" t="s">
         <v>4</v>
       </c>
@@ -1500,7 +1522,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="113" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:3">
       <c r="A113" s="2" t="s">
         <v>1</v>
       </c>
@@ -1508,7 +1530,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="114" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:3">
       <c r="A114" s="2" t="s">
         <v>2</v>
       </c>
@@ -1516,7 +1538,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="115" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:3">
       <c r="A115" s="1" t="s">
         <v>0</v>
       </c>
@@ -1524,7 +1546,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="116" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:3">
       <c r="A116" s="2" t="s">
         <v>3</v>
       </c>
@@ -1532,7 +1554,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="117" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:3">
       <c r="A117" s="2" t="s">
         <v>4</v>
       </c>
@@ -1540,7 +1562,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="119" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:3">
       <c r="A119" s="2" t="s">
         <v>1</v>
       </c>
@@ -1548,7 +1570,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="120" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="120" spans="1:3">
       <c r="A120" s="2" t="s">
         <v>2</v>
       </c>
@@ -1559,7 +1581,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="121" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:3">
       <c r="A121" s="1" t="s">
         <v>0</v>
       </c>
@@ -1567,7 +1589,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="122" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:3">
       <c r="A122" s="2" t="s">
         <v>3</v>
       </c>
@@ -1575,7 +1597,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="123" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:3">
       <c r="A123" s="2" t="s">
         <v>4</v>
       </c>
@@ -1583,10 +1605,10 @@
         <v>61</v>
       </c>
     </row>
-    <row r="124" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:3">
       <c r="A124" s="2"/>
     </row>
-    <row r="125" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="125" spans="1:3">
       <c r="A125" s="2" t="s">
         <v>1</v>
       </c>
@@ -1594,7 +1616,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="126" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="126" spans="1:3">
       <c r="A126" s="2" t="s">
         <v>2</v>
       </c>
@@ -1605,7 +1627,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="127" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="127" spans="1:3">
       <c r="A127" s="1" t="s">
         <v>0</v>
       </c>
@@ -1613,7 +1635,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="128" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="128" spans="1:3">
       <c r="A128" s="2" t="s">
         <v>3</v>
       </c>
@@ -1621,7 +1643,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="129" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="129" spans="1:2">
       <c r="A129" s="2" t="s">
         <v>4</v>
       </c>
@@ -1629,217 +1651,220 @@
         <v>61</v>
       </c>
     </row>
-    <row r="130" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="130" spans="1:2">
       <c r="A130" s="2"/>
     </row>
-    <row r="131" spans="1:2" ht="18" x14ac:dyDescent="0.2">
-      <c r="A131" s="3" t="s">
+    <row r="131" spans="1:2">
+      <c r="A131" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B131" s="7" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="132" spans="1:2">
+      <c r="A132" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B132" s="7" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="133" spans="1:2">
+      <c r="A133" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B133" s="8" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="134" spans="1:2">
+      <c r="A134" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B134" s="4" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="135" spans="1:2">
+      <c r="A135" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B135" s="4" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="136" spans="1:2">
+      <c r="A136" s="2"/>
+    </row>
+    <row r="137" spans="1:2" ht="18">
+      <c r="A137" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="132" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A132" s="2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="133" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A133" s="2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="134" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A134" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="135" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A135" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="136" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A136" s="2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="138" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="138" spans="1:2">
       <c r="A138" s="2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="139" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="139" spans="1:2">
       <c r="A139" s="2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="140" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="140" spans="1:2">
       <c r="A140" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="141" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="141" spans="1:2">
       <c r="A141" s="2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="142" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="142" spans="1:2">
       <c r="A142" s="2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="144" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="144" spans="1:2">
       <c r="A144" s="2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="145" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="145" spans="1:1">
       <c r="A145" s="2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="146" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="146" spans="1:1">
       <c r="A146" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="147" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="147" spans="1:1">
       <c r="A147" s="2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="148" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="148" spans="1:1">
       <c r="A148" s="2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="150" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="150" spans="1:1">
       <c r="A150" s="2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="151" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="151" spans="1:1">
       <c r="A151" s="2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="152" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="152" spans="1:1">
       <c r="A152" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="153" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="153" spans="1:1">
       <c r="A153" s="2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="154" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="154" spans="1:1">
       <c r="A154" s="2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="156" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="156" spans="1:1">
       <c r="A156" s="2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="157" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="157" spans="1:1">
       <c r="A157" s="2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="158" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="158" spans="1:1">
       <c r="A158" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="159" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="159" spans="1:1">
       <c r="A159" s="2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="160" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="160" spans="1:1">
       <c r="A160" s="2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="162" spans="1:2" ht="18" x14ac:dyDescent="0.2">
-      <c r="A162" s="3" t="s">
+    <row r="162" spans="1:2">
+      <c r="A162" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="163" spans="1:2">
+      <c r="A163" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="164" spans="1:2">
+      <c r="A164" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="165" spans="1:2">
+      <c r="A165" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="166" spans="1:2">
+      <c r="A166" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="168" spans="1:2" ht="18">
+      <c r="A168" s="3" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="163" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A163" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B163" s="5" t="s">
+    <row r="169" spans="1:2">
+      <c r="A169" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B169" s="5" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="164" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A164" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B164" s="5" t="s">
+    <row r="170" spans="1:2">
+      <c r="A170" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B170" s="5" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="165" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A165" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B165" s="5" t="s">
+    <row r="171" spans="1:2">
+      <c r="A171" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B171" s="5" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="166" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A166" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B166" s="4" t="s">
+    <row r="172" spans="1:2">
+      <c r="A172" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B172" s="4" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="167" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A167" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="B167" s="4" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="169" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A169" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B169" s="5" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="170" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A170" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B170" s="5" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="171" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A171" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B171" s="5" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="172" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A172" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B172" s="4" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="173" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="173" spans="1:2">
       <c r="A173" s="2" t="s">
         <v>4</v>
       </c>
@@ -1847,39 +1872,39 @@
         <v>85</v>
       </c>
     </row>
-    <row r="175" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="175" spans="1:2">
       <c r="A175" s="2" t="s">
         <v>1</v>
       </c>
       <c r="B175" s="5" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="176" spans="1:2" x14ac:dyDescent="0.2">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="176" spans="1:2">
       <c r="A176" s="2" t="s">
         <v>2</v>
       </c>
       <c r="B176" s="5" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="177" spans="1:2" x14ac:dyDescent="0.2">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="177" spans="1:2">
       <c r="A177" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B177" s="5" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="178" spans="1:2" x14ac:dyDescent="0.2">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="178" spans="1:2">
       <c r="A178" s="2" t="s">
         <v>3</v>
       </c>
       <c r="B178" s="4" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="179" spans="1:2" x14ac:dyDescent="0.2">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="179" spans="1:2">
       <c r="A179" s="2" t="s">
         <v>4</v>
       </c>
@@ -1887,39 +1912,39 @@
         <v>85</v>
       </c>
     </row>
-    <row r="181" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="181" spans="1:2">
       <c r="A181" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B181" s="6" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="182" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="B181" s="5" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="182" spans="1:2">
       <c r="A182" s="2" t="s">
         <v>2</v>
       </c>
       <c r="B182" s="5" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="183" spans="1:2" x14ac:dyDescent="0.2">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="183" spans="1:2">
       <c r="A183" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B183" s="4" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="184" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="B183" s="5" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="184" spans="1:2">
       <c r="A184" s="2" t="s">
         <v>3</v>
       </c>
       <c r="B184" s="4" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="185" spans="1:2" x14ac:dyDescent="0.2">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="185" spans="1:2">
       <c r="A185" s="2" t="s">
         <v>4</v>
       </c>
@@ -1927,43 +1952,83 @@
         <v>85</v>
       </c>
     </row>
-    <row r="187" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="187" spans="1:2">
       <c r="A187" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B187" s="5" t="s">
+      <c r="B187" s="6" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="188" spans="1:2">
+      <c r="A188" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B188" s="5" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="189" spans="1:2">
+      <c r="A189" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B189" s="4" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="190" spans="1:2">
+      <c r="A190" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B190" s="4" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="191" spans="1:2">
+      <c r="A191" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B191" s="4" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="193" spans="1:2">
+      <c r="A193" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B193" s="5" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="188" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A188" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B188" s="5" t="s">
+    <row r="194" spans="1:2">
+      <c r="A194" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B194" s="5" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="189" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A189" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B189" s="5" t="s">
+    <row r="195" spans="1:2">
+      <c r="A195" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B195" s="5" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="190" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A190" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B190" s="4" t="s">
+    <row r="196" spans="1:2">
+      <c r="A196" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B196" s="4" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="191" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A191" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="B191" s="4" t="s">
+    <row r="197" spans="1:2">
+      <c r="A197" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B197" s="4" t="s">
         <v>85</v>
       </c>
     </row>
@@ -1989,17 +2054,18 @@
     <hyperlink ref="A109" r:id="rId18" display="https://developers.google.com/maps/documentation/places/web-service/place-id" xr:uid="{91A42C1B-5438-4047-A234-D04C1C21936F}"/>
     <hyperlink ref="A115" r:id="rId19" display="https://developers.google.com/maps/documentation/places/web-service/place-id" xr:uid="{FCF31CC6-CCB4-C44C-8EF9-6907A1695F79}"/>
     <hyperlink ref="A121" r:id="rId20" display="https://developers.google.com/maps/documentation/places/web-service/place-id" xr:uid="{901E1C89-576D-C64B-955D-4A1B488F2F47}"/>
-    <hyperlink ref="A134" r:id="rId21" display="https://developers.google.com/maps/documentation/places/web-service/place-id" xr:uid="{6214FB8D-4404-8A4C-A1C6-7F93426241FD}"/>
-    <hyperlink ref="A140" r:id="rId22" display="https://developers.google.com/maps/documentation/places/web-service/place-id" xr:uid="{C6FD5ECC-C016-0443-A1AA-5D4A4C8D093D}"/>
-    <hyperlink ref="A146" r:id="rId23" display="https://developers.google.com/maps/documentation/places/web-service/place-id" xr:uid="{C2EDA595-7D76-5148-BF12-C97E8091224C}"/>
-    <hyperlink ref="A152" r:id="rId24" display="https://developers.google.com/maps/documentation/places/web-service/place-id" xr:uid="{F65090E9-270B-9441-A9A3-E95E5D8BD01C}"/>
-    <hyperlink ref="A158" r:id="rId25" display="https://developers.google.com/maps/documentation/places/web-service/place-id" xr:uid="{CE5E11BD-3C09-C54E-89E8-4652894D75CF}"/>
-    <hyperlink ref="A165" r:id="rId26" display="https://developers.google.com/maps/documentation/places/web-service/place-id" xr:uid="{B52C4AFB-E5A1-4940-B8E1-E8A6C0663DAE}"/>
-    <hyperlink ref="A171" r:id="rId27" display="https://developers.google.com/maps/documentation/places/web-service/place-id" xr:uid="{1108C462-89F4-AE4B-8FEA-2DFDBF646123}"/>
-    <hyperlink ref="A177" r:id="rId28" display="https://developers.google.com/maps/documentation/places/web-service/place-id" xr:uid="{58B520D3-90C3-3642-9CE1-77F09B4C0421}"/>
-    <hyperlink ref="A183" r:id="rId29" display="https://developers.google.com/maps/documentation/places/web-service/place-id" xr:uid="{9FB2F3E1-5A3D-A846-8375-F0831EF77342}"/>
-    <hyperlink ref="A189" r:id="rId30" display="https://developers.google.com/maps/documentation/places/web-service/place-id" xr:uid="{DE3D79FD-24A8-9B48-B76A-8C560E6D021A}"/>
+    <hyperlink ref="A140" r:id="rId21" display="https://developers.google.com/maps/documentation/places/web-service/place-id" xr:uid="{6214FB8D-4404-8A4C-A1C6-7F93426241FD}"/>
+    <hyperlink ref="A146" r:id="rId22" display="https://developers.google.com/maps/documentation/places/web-service/place-id" xr:uid="{C6FD5ECC-C016-0443-A1AA-5D4A4C8D093D}"/>
+    <hyperlink ref="A152" r:id="rId23" display="https://developers.google.com/maps/documentation/places/web-service/place-id" xr:uid="{C2EDA595-7D76-5148-BF12-C97E8091224C}"/>
+    <hyperlink ref="A158" r:id="rId24" display="https://developers.google.com/maps/documentation/places/web-service/place-id" xr:uid="{F65090E9-270B-9441-A9A3-E95E5D8BD01C}"/>
+    <hyperlink ref="A164" r:id="rId25" display="https://developers.google.com/maps/documentation/places/web-service/place-id" xr:uid="{CE5E11BD-3C09-C54E-89E8-4652894D75CF}"/>
+    <hyperlink ref="A171" r:id="rId26" display="https://developers.google.com/maps/documentation/places/web-service/place-id" xr:uid="{B52C4AFB-E5A1-4940-B8E1-E8A6C0663DAE}"/>
+    <hyperlink ref="A177" r:id="rId27" display="https://developers.google.com/maps/documentation/places/web-service/place-id" xr:uid="{1108C462-89F4-AE4B-8FEA-2DFDBF646123}"/>
+    <hyperlink ref="A183" r:id="rId28" display="https://developers.google.com/maps/documentation/places/web-service/place-id" xr:uid="{58B520D3-90C3-3642-9CE1-77F09B4C0421}"/>
+    <hyperlink ref="A189" r:id="rId29" display="https://developers.google.com/maps/documentation/places/web-service/place-id" xr:uid="{9FB2F3E1-5A3D-A846-8375-F0831EF77342}"/>
+    <hyperlink ref="A195" r:id="rId30" display="https://developers.google.com/maps/documentation/places/web-service/place-id" xr:uid="{DE3D79FD-24A8-9B48-B76A-8C560E6D021A}"/>
     <hyperlink ref="A127" r:id="rId31" display="https://developers.google.com/maps/documentation/places/web-service/place-id" xr:uid="{F2C53E2F-7B4D-CF46-BCEC-A038ACC2EE59}"/>
+    <hyperlink ref="A133" r:id="rId32" display="https://developers.google.com/maps/documentation/places/web-service/place-id" xr:uid="{20C46252-711A-634A-A49E-B6D21F5AD5A4}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>